<commit_message>
Remove obsolete government spread routes and browser fallbacks
</commit_message>
<xml_diff>
--- a/excel/ConvexDemo.xlsx
+++ b/excel/ConvexDemo.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Bonds" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Curves" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Spreads" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Scenarios" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Schemas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonds" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curves" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spreads" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schemas" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1044,7 +1044,7 @@
         <v/>
       </c>
       <c r="B19" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         <v/>
       </c>
       <c r="B20" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1136,7 +1136,7 @@
         <v/>
       </c>
       <c r="B21" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1671,7 +1671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1726,7 +1726,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="7">
@@ -1834,77 +1834,22 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>G-spread requires a separate government curve</t>
+          <t>Government spreads use actual securities</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Tenor</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Govt zero (decimal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>2</v>
-      </c>
-      <c r="B18" t="n">
-        <v>0.042</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>5</v>
-      </c>
-      <c r="B19" t="n">
-        <v>0.044</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>10</v>
-      </c>
-      <c r="B20" t="n">
-        <v>0.045</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>30</v>
-      </c>
-      <c r="B21" t="n">
-        <v>0.046</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Govt curve handle:</t>
-        </is>
-      </c>
-      <c r="B23">
-        <f>CX.CURVE("USD.TSY.DEMO",TODAY(),A18:A21,B18:B21,"zero_rate","linear","Act365Fixed","Continuous")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>G-spread today is wired only via the Spread Ticket ribbon form, which threads params.govt_curve through. The cell-side helper UDF will land in the next pass; open the ribbon Spread Ticket to compute G-spread interactively.</t>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>CX.SPREAD and the Spread Ticket cannot supply government benchmark securities. Use CX.LIBRARY.RANGE with a full government_spread request and actual cash security quotes/calendars. Government zero rates are not bond yields.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A25:F25"/>
     <mergeCell ref="A15:G15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1960,7 +1905,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Bring over the #132 workflow tree without its large fixtures
This is the final tree of codex/production-readiness-pr (#132, head
feb8e889), except for the 631 regression corpora of 1 MB or more under
tests/fixtures/library (5.91 GB, seven of them in Git LFS). The next commit
adds them back as xz archives. The code was produced by Codex and is
carried over unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/ConvexDemo.xlsx
+++ b/excel/ConvexDemo.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Bonds" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Curves" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Spreads" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Scenarios" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Schemas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonds" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curves" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spreads" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schemas" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1044,7 +1044,7 @@
         <v/>
       </c>
       <c r="B19" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         <v/>
       </c>
       <c r="B20" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1136,7 +1136,7 @@
         <v/>
       </c>
       <c r="B21" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1671,7 +1671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1726,7 +1726,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="7">
@@ -1834,77 +1834,22 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>G-spread requires a separate government curve</t>
+          <t>Government spreads use actual securities</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Tenor</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Govt zero (decimal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>2</v>
-      </c>
-      <c r="B18" t="n">
-        <v>0.042</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>5</v>
-      </c>
-      <c r="B19" t="n">
-        <v>0.044</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>10</v>
-      </c>
-      <c r="B20" t="n">
-        <v>0.045</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>30</v>
-      </c>
-      <c r="B21" t="n">
-        <v>0.046</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Govt curve handle:</t>
-        </is>
-      </c>
-      <c r="B23">
-        <f>CX.CURVE("USD.TSY.DEMO",TODAY(),A18:A21,B18:B21,"zero_rate","linear","Act365Fixed","Continuous")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>G-spread today is wired only via the Spread Ticket ribbon form, which threads params.govt_curve through. The cell-side helper UDF will land in the next pass; open the ribbon Spread Ticket to compute G-spread interactively.</t>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>CX.SPREAD and the Spread Ticket cannot supply government benchmark securities. Use CX.LIBRARY.RANGE with a full government_spread request and actual cash security quotes/calendars. Government zero rates are not bond yields.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A25:F25"/>
     <mergeCell ref="A15:G15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1960,7 +1905,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Replace #132: pack fixtures, fix CI, remove hash pinning (#133)
</commit_message>
<xml_diff>
--- a/excel/ConvexDemo.xlsx
+++ b/excel/ConvexDemo.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Bonds" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Curves" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Spreads" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Scenarios" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Schemas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonds" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curves" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spreads" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schemas" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1044,7 +1044,7 @@
         <v/>
       </c>
       <c r="B19" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         <v/>
       </c>
       <c r="B20" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1136,7 +1136,7 @@
         <v/>
       </c>
       <c r="B21" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1671,7 +1671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1726,7 +1726,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="7">
@@ -1834,77 +1834,22 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>G-spread requires a separate government curve</t>
+          <t>Government spreads use actual securities</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Tenor</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Govt zero (decimal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>2</v>
-      </c>
-      <c r="B18" t="n">
-        <v>0.042</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>5</v>
-      </c>
-      <c r="B19" t="n">
-        <v>0.044</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>10</v>
-      </c>
-      <c r="B20" t="n">
-        <v>0.045</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>30</v>
-      </c>
-      <c r="B21" t="n">
-        <v>0.046</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Govt curve handle:</t>
-        </is>
-      </c>
-      <c r="B23">
-        <f>CX.CURVE("USD.TSY.DEMO",TODAY(),A18:A21,B18:B21,"zero_rate","linear","Act365Fixed","Continuous")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>G-spread today is wired only via the Spread Ticket ribbon form, which threads params.govt_curve through. The cell-side helper UDF will land in the next pass; open the ribbon Spread Ticket to compute G-spread interactively.</t>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>CX.SPREAD and the Spread Ticket cannot supply government benchmark securities. Use CX.LIBRARY.RANGE with a full government_spread request and actual cash security quotes/calendars. Government zero rates are not bond yields.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A25:F25"/>
     <mergeCell ref="A15:G15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1960,7 +1905,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>46140</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="6">

</xml_diff>